<commit_message>
added TOC and Project Ideas
</commit_message>
<xml_diff>
--- a/My leaning Roadmap and Tracker.xlsx
+++ b/My leaning Roadmap and Tracker.xlsx
@@ -1,14 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28029"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="255" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A671C1D-99EE-4C7C-B276-61D262438A21}"/>
+  <xr:revisionPtr revIDLastSave="307" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31F3AE7F-93E1-4E2A-BD83-66009D208BAE}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Roadmap" sheetId="1" r:id="rId1"/>
+    <sheet name="TOC" sheetId="2" r:id="rId2"/>
+    <sheet name="Project Ideas" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -31,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="98">
   <si>
     <r>
       <rPr>
@@ -320,12 +322,213 @@
   <si>
     <t>Python 3 Object-Oriented Programming E3</t>
   </si>
+  <si>
+    <t>Table of Content</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Fundamentals</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>Programming Conceps</t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
+    <t>Syntax &amp; Semantics</t>
+  </si>
+  <si>
+    <t>ii</t>
+  </si>
+  <si>
+    <t>Variables</t>
+  </si>
+  <si>
+    <t>iii</t>
+  </si>
+  <si>
+    <t>Data Types</t>
+  </si>
+  <si>
+    <t>iv</t>
+  </si>
+  <si>
+    <t>Expressions &amp; Operators</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>Keywords</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>Control Structure &amp; Flow</t>
+  </si>
+  <si>
+    <t>If-Else statements</t>
+  </si>
+  <si>
+    <t>Loops (for, do, do-while, while)</t>
+  </si>
+  <si>
+    <t>Switch-Case statements</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>Functions</t>
+  </si>
+  <si>
+    <t>Understand Parameter &amp; Arguments</t>
+  </si>
+  <si>
+    <t>Return Types</t>
+  </si>
+  <si>
+    <t>Scope</t>
+  </si>
+  <si>
+    <t>Higher-Order Functions</t>
+  </si>
+  <si>
+    <t>Lambda expressions</t>
+  </si>
+  <si>
+    <t>vi</t>
+  </si>
+  <si>
+    <t>Immutability</t>
+  </si>
+  <si>
+    <t>Data Structures</t>
+  </si>
+  <si>
+    <t>Arrays &amp; Lists</t>
+  </si>
+  <si>
+    <t>Stacks &amp; Queues</t>
+  </si>
+  <si>
+    <t>Linked Lists</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>Dictionaries &amp; Hashmaps</t>
+  </si>
+  <si>
+    <t>e</t>
+  </si>
+  <si>
+    <t>Trees &amp; Graphs</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
+  <si>
+    <t>Strings</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
+    <t>Tuples</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>Sets &amp; Maps</t>
+  </si>
+  <si>
+    <t>Algorithms</t>
+  </si>
+  <si>
+    <t>Searching &amp; Sorting</t>
+  </si>
+  <si>
+    <t>Recursion</t>
+  </si>
+  <si>
+    <t>Complexity Analysis</t>
+  </si>
+  <si>
+    <t>Object-Oriented Programming</t>
+  </si>
+  <si>
+    <t>Classes and Objects</t>
+  </si>
+  <si>
+    <t>Inheritance</t>
+  </si>
+  <si>
+    <t>Polymorphism</t>
+  </si>
+  <si>
+    <t>Encapsulation</t>
+  </si>
+  <si>
+    <t>Abstraction</t>
+  </si>
+  <si>
+    <t>Magic methods</t>
+  </si>
+  <si>
+    <t>Operator overloading</t>
+  </si>
+  <si>
+    <t>Error Handling and Debugging</t>
+  </si>
+  <si>
+    <t>Exceptions</t>
+  </si>
+  <si>
+    <t>Debugging Techniques and Tools</t>
+  </si>
+  <si>
+    <t>Working with Files</t>
+  </si>
+  <si>
+    <t>Files I/O</t>
+  </si>
+  <si>
+    <t>Extra</t>
+  </si>
+  <si>
+    <t>Regular Expressions</t>
+  </si>
+  <si>
+    <t>Date and Time</t>
+  </si>
+  <si>
+    <t>No.</t>
+  </si>
+  <si>
+    <t>Ideas</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Work progress tracker</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -403,8 +606,21 @@
       <color rgb="FFFF1B6B"/>
       <name val="Arial Black"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Sylfaen"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Sylfaen"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -459,6 +675,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="45">
     <border>
@@ -1028,7 +1250,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1046,89 +1268,47 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1138,13 +1318,23 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1155,56 +1345,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1217,17 +1357,156 @@
     <xf numFmtId="0" fontId="10" fillId="9" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1236,16 +1515,16 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <colors>
     <mruColors>
-      <color rgb="FF07F49E"/>
-      <color rgb="FFFDFFB6"/>
       <color rgb="FFFF1B6B"/>
-      <color rgb="FF42047E"/>
       <color rgb="FFCAFFBF"/>
       <color rgb="FFFFADAD"/>
       <color rgb="FFBDB2FF"/>
+      <color rgb="FF9BF6FF"/>
       <color rgb="FFA0C4FF"/>
-      <color rgb="FF9BF6FF"/>
       <color rgb="FFFFD6A5"/>
+      <color rgb="FF07F49E"/>
+      <color rgb="FFFDFFB6"/>
+      <color rgb="FF42047E"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1586,103 +1865,103 @@
   <sheetData>
     <row r="1" spans="1:45" ht="15" customHeight="1">
       <c r="A1" s="4"/>
-      <c r="B1" s="76" t="s">
+      <c r="B1" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="77"/>
-      <c r="J1" s="77"/>
-      <c r="K1" s="77"/>
-      <c r="L1" s="77"/>
-      <c r="M1" s="77"/>
-      <c r="N1" s="77"/>
-      <c r="O1" s="77"/>
-      <c r="P1" s="77"/>
-      <c r="Q1" s="77"/>
-      <c r="R1" s="77"/>
-      <c r="S1" s="77"/>
-      <c r="T1" s="77"/>
-      <c r="U1" s="77"/>
-      <c r="V1" s="77"/>
-      <c r="W1" s="77"/>
-      <c r="X1" s="77"/>
-      <c r="Y1" s="77"/>
-      <c r="Z1" s="77"/>
-      <c r="AA1" s="77"/>
-      <c r="AB1" s="77"/>
-      <c r="AC1" s="77"/>
-      <c r="AD1" s="77"/>
-      <c r="AE1" s="77"/>
-      <c r="AF1" s="77"/>
-      <c r="AG1" s="77"/>
-      <c r="AH1" s="77"/>
-      <c r="AI1" s="77"/>
-      <c r="AJ1" s="77"/>
-      <c r="AK1" s="77"/>
-      <c r="AL1" s="77"/>
-      <c r="AM1" s="77"/>
-      <c r="AN1" s="77"/>
-      <c r="AO1" s="77"/>
-      <c r="AP1" s="77"/>
-      <c r="AQ1" s="77"/>
-      <c r="AR1" s="78"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
+      <c r="L1" s="55"/>
+      <c r="M1" s="55"/>
+      <c r="N1" s="55"/>
+      <c r="O1" s="55"/>
+      <c r="P1" s="55"/>
+      <c r="Q1" s="55"/>
+      <c r="R1" s="55"/>
+      <c r="S1" s="55"/>
+      <c r="T1" s="55"/>
+      <c r="U1" s="55"/>
+      <c r="V1" s="55"/>
+      <c r="W1" s="55"/>
+      <c r="X1" s="55"/>
+      <c r="Y1" s="55"/>
+      <c r="Z1" s="55"/>
+      <c r="AA1" s="55"/>
+      <c r="AB1" s="55"/>
+      <c r="AC1" s="55"/>
+      <c r="AD1" s="55"/>
+      <c r="AE1" s="55"/>
+      <c r="AF1" s="55"/>
+      <c r="AG1" s="55"/>
+      <c r="AH1" s="55"/>
+      <c r="AI1" s="55"/>
+      <c r="AJ1" s="55"/>
+      <c r="AK1" s="55"/>
+      <c r="AL1" s="55"/>
+      <c r="AM1" s="55"/>
+      <c r="AN1" s="55"/>
+      <c r="AO1" s="55"/>
+      <c r="AP1" s="55"/>
+      <c r="AQ1" s="55"/>
+      <c r="AR1" s="56"/>
       <c r="AS1" s="5"/>
     </row>
     <row r="2" spans="1:45" ht="15" customHeight="1">
-      <c r="A2" s="74"/>
-      <c r="B2" s="79"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="19"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="19"/>
-      <c r="V2" s="19"/>
-      <c r="W2" s="19"/>
-      <c r="X2" s="19"/>
-      <c r="Y2" s="19"/>
-      <c r="Z2" s="19"/>
-      <c r="AA2" s="19"/>
-      <c r="AB2" s="19"/>
-      <c r="AC2" s="19"/>
-      <c r="AD2" s="19"/>
-      <c r="AE2" s="19"/>
-      <c r="AF2" s="19"/>
-      <c r="AG2" s="19"/>
-      <c r="AH2" s="19"/>
-      <c r="AI2" s="19"/>
-      <c r="AJ2" s="19"/>
-      <c r="AK2" s="19"/>
-      <c r="AL2" s="19"/>
-      <c r="AM2" s="19"/>
-      <c r="AN2" s="19"/>
-      <c r="AO2" s="19"/>
-      <c r="AP2" s="19"/>
-      <c r="AQ2" s="19"/>
-      <c r="AR2" s="80"/>
+      <c r="A2" s="26"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
+      <c r="L2" s="58"/>
+      <c r="M2" s="58"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="58"/>
+      <c r="P2" s="58"/>
+      <c r="Q2" s="58"/>
+      <c r="R2" s="58"/>
+      <c r="S2" s="58"/>
+      <c r="T2" s="58"/>
+      <c r="U2" s="58"/>
+      <c r="V2" s="58"/>
+      <c r="W2" s="58"/>
+      <c r="X2" s="58"/>
+      <c r="Y2" s="58"/>
+      <c r="Z2" s="58"/>
+      <c r="AA2" s="58"/>
+      <c r="AB2" s="58"/>
+      <c r="AC2" s="58"/>
+      <c r="AD2" s="58"/>
+      <c r="AE2" s="58"/>
+      <c r="AF2" s="58"/>
+      <c r="AG2" s="58"/>
+      <c r="AH2" s="58"/>
+      <c r="AI2" s="58"/>
+      <c r="AJ2" s="58"/>
+      <c r="AK2" s="58"/>
+      <c r="AL2" s="58"/>
+      <c r="AM2" s="58"/>
+      <c r="AN2" s="58"/>
+      <c r="AO2" s="58"/>
+      <c r="AP2" s="58"/>
+      <c r="AQ2" s="58"/>
+      <c r="AR2" s="59"/>
       <c r="AS2" s="5"/>
     </row>
     <row r="3" spans="1:45" ht="15.75" customHeight="1">
-      <c r="A3" s="72"/>
-      <c r="B3" s="81"/>
+      <c r="A3" s="24"/>
+      <c r="B3" s="28"/>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -1719,112 +1998,112 @@
       <c r="AJ3" s="7"/>
       <c r="AK3" s="7"/>
       <c r="AL3" s="2"/>
-      <c r="AM3" s="33"/>
-      <c r="AN3" s="33"/>
-      <c r="AO3" s="33"/>
-      <c r="AP3" s="33"/>
-      <c r="AQ3" s="33"/>
-      <c r="AR3" s="82"/>
+      <c r="AM3" s="15"/>
+      <c r="AN3" s="15"/>
+      <c r="AO3" s="15"/>
+      <c r="AP3" s="15"/>
+      <c r="AQ3" s="15"/>
+      <c r="AR3" s="29"/>
       <c r="AS3" s="5"/>
     </row>
     <row r="4" spans="1:45" ht="17.25">
       <c r="A4" s="11"/>
-      <c r="B4" s="83"/>
-      <c r="C4" s="35" t="s">
+      <c r="B4" s="30"/>
+      <c r="C4" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="37"/>
+      <c r="D4" s="69"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="70"/>
       <c r="H4" s="5"/>
-      <c r="I4" s="17" t="s">
+      <c r="I4" s="60" t="s">
         <v>2</v>
       </c>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
+      <c r="J4" s="61"/>
+      <c r="K4" s="61"/>
+      <c r="L4" s="61"/>
+      <c r="M4" s="61"/>
       <c r="N4" s="4"/>
-      <c r="O4" s="21" t="s">
+      <c r="O4" s="62" t="s">
         <v>3</v>
       </c>
-      <c r="P4" s="22"/>
-      <c r="Q4" s="22"/>
-      <c r="R4" s="22"/>
-      <c r="S4" s="23"/>
+      <c r="P4" s="63"/>
+      <c r="Q4" s="63"/>
+      <c r="R4" s="63"/>
+      <c r="S4" s="64"/>
       <c r="T4" s="10"/>
-      <c r="U4" s="54" t="s">
+      <c r="U4" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="V4" s="55"/>
-      <c r="W4" s="55"/>
-      <c r="X4" s="55"/>
-      <c r="Y4" s="56"/>
+      <c r="V4" s="66"/>
+      <c r="W4" s="66"/>
+      <c r="X4" s="66"/>
+      <c r="Y4" s="67"/>
       <c r="Z4" s="11"/>
-      <c r="AA4" s="59" t="s">
+      <c r="AA4" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="AB4" s="60"/>
-      <c r="AC4" s="60"/>
-      <c r="AD4" s="60"/>
-      <c r="AE4" s="61"/>
+      <c r="AB4" s="75"/>
+      <c r="AC4" s="75"/>
+      <c r="AD4" s="75"/>
+      <c r="AE4" s="76"/>
       <c r="AF4" s="11"/>
-      <c r="AG4" s="65" t="s">
+      <c r="AG4" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="AH4" s="66"/>
-      <c r="AI4" s="66"/>
-      <c r="AJ4" s="66"/>
-      <c r="AK4" s="67"/>
+      <c r="AH4" s="78"/>
+      <c r="AI4" s="78"/>
+      <c r="AJ4" s="78"/>
+      <c r="AK4" s="79"/>
       <c r="AL4" s="11"/>
-      <c r="AM4" s="68" t="s">
+      <c r="AM4" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="AN4" s="69"/>
-      <c r="AO4" s="69"/>
-      <c r="AP4" s="69"/>
-      <c r="AQ4" s="70"/>
-      <c r="AR4" s="84"/>
+      <c r="AN4" s="72"/>
+      <c r="AO4" s="72"/>
+      <c r="AP4" s="72"/>
+      <c r="AQ4" s="73"/>
+      <c r="AR4" s="31"/>
       <c r="AS4" s="5"/>
     </row>
     <row r="5" spans="1:45">
       <c r="A5" s="11"/>
-      <c r="B5" s="83"/>
-      <c r="C5" s="24"/>
-      <c r="G5" s="25"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="13"/>
+      <c r="G5" s="14"/>
       <c r="H5" s="5"/>
       <c r="N5" s="4"/>
-      <c r="O5" s="47"/>
-      <c r="P5" s="33"/>
-      <c r="Q5" s="33"/>
-      <c r="R5" s="33"/>
-      <c r="S5" s="48"/>
+      <c r="O5" s="18"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
+      <c r="R5" s="15"/>
+      <c r="S5" s="19"/>
       <c r="T5" s="11"/>
-      <c r="U5" s="24"/>
-      <c r="Y5" s="25"/>
+      <c r="U5" s="13"/>
+      <c r="Y5" s="14"/>
       <c r="Z5" s="11"/>
-      <c r="AA5" s="24"/>
-      <c r="AE5" s="25"/>
+      <c r="AA5" s="13"/>
+      <c r="AE5" s="14"/>
       <c r="AF5" s="11"/>
-      <c r="AG5" s="24"/>
-      <c r="AK5" s="25"/>
+      <c r="AG5" s="13"/>
+      <c r="AK5" s="14"/>
       <c r="AL5" s="11"/>
-      <c r="AM5" s="24"/>
-      <c r="AQ5" s="25"/>
-      <c r="AR5" s="84"/>
+      <c r="AM5" s="13"/>
+      <c r="AQ5" s="14"/>
+      <c r="AR5" s="31"/>
       <c r="AS5" s="5"/>
     </row>
     <row r="6" spans="1:45" ht="15.75">
       <c r="A6" s="11"/>
-      <c r="B6" s="83"/>
-      <c r="C6" s="26" t="s">
+      <c r="B6" s="30"/>
+      <c r="C6" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="27"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="38"/>
       <c r="H6" s="6"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
@@ -1832,58 +2111,58 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
       <c r="N6" s="9"/>
-      <c r="O6" s="30" t="s">
+      <c r="O6" s="80" t="s">
         <v>9</v>
       </c>
-      <c r="P6" s="31"/>
-      <c r="Q6" s="31"/>
-      <c r="R6" s="31"/>
-      <c r="S6" s="32"/>
+      <c r="P6" s="81"/>
+      <c r="Q6" s="81"/>
+      <c r="R6" s="81"/>
+      <c r="S6" s="82"/>
       <c r="T6" s="12"/>
-      <c r="U6" s="26" t="s">
+      <c r="U6" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="V6" s="13"/>
-      <c r="W6" s="13"/>
-      <c r="X6" s="13"/>
-      <c r="Y6" s="27"/>
+      <c r="V6" s="37"/>
+      <c r="W6" s="37"/>
+      <c r="X6" s="37"/>
+      <c r="Y6" s="38"/>
       <c r="Z6" s="12"/>
-      <c r="AA6" s="26" t="s">
+      <c r="AA6" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="AB6" s="13"/>
-      <c r="AC6" s="13"/>
-      <c r="AD6" s="13"/>
-      <c r="AE6" s="27"/>
+      <c r="AB6" s="37"/>
+      <c r="AC6" s="37"/>
+      <c r="AD6" s="37"/>
+      <c r="AE6" s="38"/>
       <c r="AF6" s="12"/>
-      <c r="AG6" s="26" t="s">
+      <c r="AG6" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="AH6" s="13"/>
-      <c r="AI6" s="13"/>
-      <c r="AJ6" s="13"/>
-      <c r="AK6" s="27"/>
+      <c r="AH6" s="37"/>
+      <c r="AI6" s="37"/>
+      <c r="AJ6" s="37"/>
+      <c r="AK6" s="38"/>
       <c r="AL6" s="11"/>
-      <c r="AM6" s="26" t="s">
+      <c r="AM6" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="AN6" s="13"/>
-      <c r="AO6" s="13"/>
-      <c r="AP6" s="13"/>
-      <c r="AQ6" s="27"/>
-      <c r="AR6" s="84"/>
+      <c r="AN6" s="37"/>
+      <c r="AO6" s="37"/>
+      <c r="AP6" s="37"/>
+      <c r="AQ6" s="38"/>
+      <c r="AR6" s="31"/>
       <c r="AS6" s="5"/>
     </row>
     <row r="7" spans="1:45" ht="15.75">
       <c r="A7" s="11"/>
-      <c r="B7" s="83"/>
-      <c r="C7" s="38" t="s">
+      <c r="B7" s="30"/>
+      <c r="C7" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="39"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
+      <c r="G7" s="47"/>
       <c r="H7" s="6"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
@@ -1891,58 +2170,58 @@
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
       <c r="N7" s="9"/>
-      <c r="O7" s="28" t="s">
+      <c r="O7" s="83" t="s">
         <v>12</v>
       </c>
-      <c r="P7" s="16"/>
-      <c r="Q7" s="16"/>
-      <c r="R7" s="16"/>
-      <c r="S7" s="29"/>
+      <c r="P7" s="84"/>
+      <c r="Q7" s="84"/>
+      <c r="R7" s="84"/>
+      <c r="S7" s="85"/>
       <c r="T7" s="12"/>
-      <c r="U7" s="57" t="s">
+      <c r="U7" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="V7" s="15"/>
-      <c r="W7" s="15"/>
-      <c r="X7" s="15"/>
-      <c r="Y7" s="58"/>
+      <c r="V7" s="40"/>
+      <c r="W7" s="40"/>
+      <c r="X7" s="40"/>
+      <c r="Y7" s="41"/>
       <c r="Z7" s="12"/>
-      <c r="AA7" s="42" t="s">
+      <c r="AA7" s="16" t="s">
         <v>14</v>
       </c>
       <c r="AB7" s="3"/>
       <c r="AC7" s="3"/>
       <c r="AD7" s="3"/>
-      <c r="AE7" s="43"/>
+      <c r="AE7" s="17"/>
       <c r="AF7" s="12"/>
-      <c r="AG7" s="44" t="s">
+      <c r="AG7" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="AH7" s="45"/>
-      <c r="AI7" s="45"/>
-      <c r="AJ7" s="45"/>
-      <c r="AK7" s="46"/>
+      <c r="AH7" s="43"/>
+      <c r="AI7" s="43"/>
+      <c r="AJ7" s="43"/>
+      <c r="AK7" s="44"/>
       <c r="AL7" s="11"/>
-      <c r="AM7" s="57" t="s">
+      <c r="AM7" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="AN7" s="15"/>
-      <c r="AO7" s="15"/>
-      <c r="AP7" s="15"/>
-      <c r="AQ7" s="58"/>
-      <c r="AR7" s="84"/>
+      <c r="AN7" s="40"/>
+      <c r="AO7" s="40"/>
+      <c r="AP7" s="40"/>
+      <c r="AQ7" s="41"/>
+      <c r="AR7" s="31"/>
       <c r="AS7" s="5"/>
     </row>
     <row r="8" spans="1:45" ht="15.75">
       <c r="A8" s="11"/>
-      <c r="B8" s="83"/>
-      <c r="C8" s="40" t="s">
+      <c r="B8" s="30"/>
+      <c r="C8" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="41"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="49"/>
+      <c r="F8" s="49"/>
+      <c r="G8" s="50"/>
       <c r="H8" s="6"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
@@ -1950,27 +2229,27 @@
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
       <c r="N8" s="9"/>
-      <c r="O8" s="49"/>
-      <c r="P8" s="34"/>
-      <c r="Q8" s="34"/>
-      <c r="R8" s="34"/>
-      <c r="S8" s="50"/>
+      <c r="O8" s="86"/>
+      <c r="P8" s="87"/>
+      <c r="Q8" s="87"/>
+      <c r="R8" s="87"/>
+      <c r="S8" s="88"/>
       <c r="T8" s="12"/>
-      <c r="U8" s="57" t="s">
+      <c r="U8" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="V8" s="15"/>
-      <c r="W8" s="15"/>
-      <c r="X8" s="15"/>
-      <c r="Y8" s="58"/>
+      <c r="V8" s="40"/>
+      <c r="W8" s="40"/>
+      <c r="X8" s="40"/>
+      <c r="Y8" s="41"/>
       <c r="Z8" s="12"/>
-      <c r="AA8" s="42" t="s">
+      <c r="AA8" s="16" t="s">
         <v>19</v>
       </c>
       <c r="AB8" s="3"/>
       <c r="AC8" s="3"/>
       <c r="AD8" s="3"/>
-      <c r="AE8" s="43"/>
+      <c r="AE8" s="17"/>
       <c r="AF8" s="6"/>
       <c r="AG8" s="8"/>
       <c r="AH8" s="8"/>
@@ -1978,24 +2257,24 @@
       <c r="AJ8" s="8"/>
       <c r="AK8" s="8"/>
       <c r="AL8" s="4"/>
-      <c r="AM8" s="57" t="s">
+      <c r="AM8" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="AN8" s="15"/>
-      <c r="AO8" s="15"/>
-      <c r="AP8" s="15"/>
-      <c r="AQ8" s="58"/>
-      <c r="AR8" s="84"/>
+      <c r="AN8" s="40"/>
+      <c r="AO8" s="40"/>
+      <c r="AP8" s="40"/>
+      <c r="AQ8" s="41"/>
+      <c r="AR8" s="31"/>
       <c r="AS8" s="5"/>
     </row>
     <row r="9" spans="1:45" ht="15.75">
       <c r="A9" s="11"/>
-      <c r="B9" s="83"/>
-      <c r="C9" s="42"/>
+      <c r="B9" s="30"/>
+      <c r="C9" s="16"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
-      <c r="G9" s="43"/>
+      <c r="G9" s="17"/>
       <c r="H9" s="6"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -2011,19 +2290,19 @@
       <c r="R9" s="52"/>
       <c r="S9" s="53"/>
       <c r="T9" s="12"/>
-      <c r="U9" s="44" t="s">
+      <c r="U9" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="V9" s="45"/>
-      <c r="W9" s="45"/>
-      <c r="X9" s="45"/>
-      <c r="Y9" s="46"/>
+      <c r="V9" s="43"/>
+      <c r="W9" s="43"/>
+      <c r="X9" s="43"/>
+      <c r="Y9" s="44"/>
       <c r="Z9" s="12"/>
-      <c r="AA9" s="42"/>
+      <c r="AA9" s="16"/>
       <c r="AB9" s="3"/>
       <c r="AC9" s="3"/>
       <c r="AD9" s="3"/>
-      <c r="AE9" s="43"/>
+      <c r="AE9" s="17"/>
       <c r="AF9" s="6"/>
       <c r="AG9" s="3"/>
       <c r="AH9" s="3"/>
@@ -2031,26 +2310,26 @@
       <c r="AJ9" s="3"/>
       <c r="AK9" s="3"/>
       <c r="AL9" s="4"/>
-      <c r="AM9" s="44" t="s">
+      <c r="AM9" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="AN9" s="45"/>
-      <c r="AO9" s="45"/>
-      <c r="AP9" s="45"/>
-      <c r="AQ9" s="46"/>
-      <c r="AR9" s="84"/>
+      <c r="AN9" s="43"/>
+      <c r="AO9" s="43"/>
+      <c r="AP9" s="43"/>
+      <c r="AQ9" s="44"/>
+      <c r="AR9" s="31"/>
       <c r="AS9" s="5"/>
     </row>
     <row r="10" spans="1:45" ht="15.75">
       <c r="A10" s="11"/>
-      <c r="B10" s="83"/>
-      <c r="C10" s="26" t="s">
+      <c r="B10" s="30"/>
+      <c r="C10" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="27"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="37"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="38"/>
       <c r="H10" s="6"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
@@ -2070,13 +2349,13 @@
       <c r="X10" s="8"/>
       <c r="Y10" s="8"/>
       <c r="Z10" s="9"/>
-      <c r="AA10" s="26" t="s">
+      <c r="AA10" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="AB10" s="13"/>
-      <c r="AC10" s="13"/>
-      <c r="AD10" s="13"/>
-      <c r="AE10" s="27"/>
+      <c r="AB10" s="37"/>
+      <c r="AC10" s="37"/>
+      <c r="AD10" s="37"/>
+      <c r="AE10" s="38"/>
       <c r="AF10" s="6"/>
       <c r="AG10" s="3"/>
       <c r="AH10" s="3"/>
@@ -2088,19 +2367,19 @@
       <c r="AO10" s="8"/>
       <c r="AP10" s="8"/>
       <c r="AQ10" s="8"/>
-      <c r="AR10" s="82"/>
+      <c r="AR10" s="29"/>
       <c r="AS10" s="5"/>
     </row>
     <row r="11" spans="1:45" ht="15.75">
       <c r="A11" s="11"/>
-      <c r="B11" s="83"/>
-      <c r="C11" s="40" t="s">
+      <c r="B11" s="30"/>
+      <c r="C11" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="41"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49"/>
+      <c r="G11" s="50"/>
       <c r="H11" s="6"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
@@ -2120,13 +2399,13 @@
       <c r="X11" s="3"/>
       <c r="Y11" s="3"/>
       <c r="Z11" s="9"/>
-      <c r="AA11" s="62" t="s">
+      <c r="AA11" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="AB11" s="63"/>
-      <c r="AC11" s="63"/>
-      <c r="AD11" s="63"/>
-      <c r="AE11" s="64"/>
+      <c r="AB11" s="21"/>
+      <c r="AC11" s="21"/>
+      <c r="AD11" s="21"/>
+      <c r="AE11" s="22"/>
       <c r="AF11" s="6"/>
       <c r="AG11" s="3"/>
       <c r="AH11" s="3"/>
@@ -2138,19 +2417,19 @@
       <c r="AO11" s="3"/>
       <c r="AP11" s="3"/>
       <c r="AQ11" s="3"/>
-      <c r="AR11" s="82"/>
+      <c r="AR11" s="29"/>
       <c r="AS11" s="5"/>
     </row>
     <row r="12" spans="1:45" ht="15.75">
       <c r="A12" s="11"/>
-      <c r="B12" s="83"/>
-      <c r="C12" s="40" t="s">
+      <c r="B12" s="30"/>
+      <c r="C12" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="41"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="49"/>
+      <c r="F12" s="49"/>
+      <c r="G12" s="50"/>
       <c r="H12" s="6"/>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
@@ -2186,19 +2465,19 @@
       <c r="AO12" s="3"/>
       <c r="AP12" s="3"/>
       <c r="AQ12" s="3"/>
-      <c r="AR12" s="82"/>
+      <c r="AR12" s="29"/>
       <c r="AS12" s="5"/>
     </row>
     <row r="13" spans="1:45" ht="15.75">
       <c r="A13" s="11"/>
-      <c r="B13" s="83"/>
-      <c r="C13" s="40" t="s">
+      <c r="B13" s="30"/>
+      <c r="C13" s="48" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="41"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49"/>
+      <c r="G13" s="50"/>
       <c r="H13" s="6"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
@@ -2234,19 +2513,19 @@
       <c r="AO13" s="3"/>
       <c r="AP13" s="3"/>
       <c r="AQ13" s="3"/>
-      <c r="AR13" s="82"/>
+      <c r="AR13" s="29"/>
       <c r="AS13" s="5"/>
     </row>
     <row r="14" spans="1:45" ht="15.75">
       <c r="A14" s="11"/>
-      <c r="B14" s="83"/>
-      <c r="C14" s="44" t="s">
+      <c r="B14" s="30"/>
+      <c r="C14" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="46"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="43"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="44"/>
       <c r="H14" s="6"/>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
@@ -2282,12 +2561,12 @@
       <c r="AO14" s="3"/>
       <c r="AP14" s="3"/>
       <c r="AQ14" s="3"/>
-      <c r="AR14" s="82"/>
+      <c r="AR14" s="29"/>
       <c r="AS14" s="5"/>
     </row>
     <row r="15" spans="1:45" ht="15.75">
       <c r="A15" s="11"/>
-      <c r="B15" s="81"/>
+      <c r="B15" s="28"/>
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
@@ -2328,12 +2607,12 @@
       <c r="AO15" s="3"/>
       <c r="AP15" s="3"/>
       <c r="AQ15" s="3"/>
-      <c r="AR15" s="82"/>
+      <c r="AR15" s="29"/>
       <c r="AS15" s="5"/>
     </row>
     <row r="16" spans="1:45" ht="15.75">
       <c r="A16" s="11"/>
-      <c r="B16" s="81"/>
+      <c r="B16" s="28"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
@@ -2374,12 +2653,12 @@
       <c r="AO16" s="3"/>
       <c r="AP16" s="3"/>
       <c r="AQ16" s="3"/>
-      <c r="AR16" s="82"/>
+      <c r="AR16" s="29"/>
       <c r="AS16" s="5"/>
     </row>
     <row r="17" spans="1:45" ht="15.75">
       <c r="A17" s="11"/>
-      <c r="B17" s="81"/>
+      <c r="B17" s="28"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
@@ -2420,12 +2699,12 @@
       <c r="AO17" s="3"/>
       <c r="AP17" s="3"/>
       <c r="AQ17" s="3"/>
-      <c r="AR17" s="82"/>
+      <c r="AR17" s="29"/>
       <c r="AS17" s="5"/>
     </row>
     <row r="18" spans="1:45" ht="15.75">
-      <c r="A18" s="75"/>
-      <c r="B18" s="81"/>
+      <c r="A18" s="27"/>
+      <c r="B18" s="28"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
@@ -2466,12 +2745,12 @@
       <c r="AO18" s="3"/>
       <c r="AP18" s="3"/>
       <c r="AQ18" s="3"/>
-      <c r="AR18" s="82"/>
+      <c r="AR18" s="29"/>
       <c r="AS18" s="5"/>
     </row>
     <row r="19" spans="1:45" ht="15.75">
       <c r="A19" s="4"/>
-      <c r="B19" s="81"/>
+      <c r="B19" s="28"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
@@ -2512,58 +2791,58 @@
       <c r="AO19" s="3"/>
       <c r="AP19" s="3"/>
       <c r="AQ19" s="3"/>
-      <c r="AR19" s="82"/>
+      <c r="AR19" s="29"/>
       <c r="AS19" s="5"/>
     </row>
     <row r="20" spans="1:45" ht="15.75">
       <c r="A20" s="4"/>
-      <c r="B20" s="85"/>
-      <c r="C20" s="86"/>
-      <c r="D20" s="86"/>
-      <c r="E20" s="86"/>
-      <c r="F20" s="86"/>
-      <c r="G20" s="86"/>
-      <c r="H20" s="86"/>
-      <c r="I20" s="86"/>
-      <c r="J20" s="86"/>
-      <c r="K20" s="86"/>
-      <c r="L20" s="86"/>
-      <c r="M20" s="86"/>
-      <c r="N20" s="86"/>
-      <c r="O20" s="86"/>
-      <c r="P20" s="86"/>
-      <c r="Q20" s="86"/>
-      <c r="R20" s="86"/>
-      <c r="S20" s="86"/>
-      <c r="T20" s="86"/>
-      <c r="U20" s="86"/>
-      <c r="V20" s="86"/>
-      <c r="W20" s="86"/>
-      <c r="X20" s="86"/>
-      <c r="Y20" s="86"/>
-      <c r="Z20" s="86"/>
-      <c r="AA20" s="86"/>
-      <c r="AB20" s="86"/>
-      <c r="AC20" s="86"/>
-      <c r="AD20" s="86"/>
-      <c r="AE20" s="86"/>
-      <c r="AF20" s="86"/>
-      <c r="AG20" s="86"/>
-      <c r="AH20" s="86"/>
-      <c r="AI20" s="86"/>
-      <c r="AJ20" s="86"/>
-      <c r="AK20" s="86"/>
-      <c r="AL20" s="87"/>
-      <c r="AM20" s="86"/>
-      <c r="AN20" s="86"/>
-      <c r="AO20" s="86"/>
-      <c r="AP20" s="86"/>
-      <c r="AQ20" s="86"/>
-      <c r="AR20" s="88"/>
+      <c r="B20" s="32"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="33"/>
+      <c r="J20" s="33"/>
+      <c r="K20" s="33"/>
+      <c r="L20" s="33"/>
+      <c r="M20" s="33"/>
+      <c r="N20" s="33"/>
+      <c r="O20" s="33"/>
+      <c r="P20" s="33"/>
+      <c r="Q20" s="33"/>
+      <c r="R20" s="33"/>
+      <c r="S20" s="33"/>
+      <c r="T20" s="33"/>
+      <c r="U20" s="33"/>
+      <c r="V20" s="33"/>
+      <c r="W20" s="33"/>
+      <c r="X20" s="33"/>
+      <c r="Y20" s="33"/>
+      <c r="Z20" s="33"/>
+      <c r="AA20" s="33"/>
+      <c r="AB20" s="33"/>
+      <c r="AC20" s="33"/>
+      <c r="AD20" s="33"/>
+      <c r="AE20" s="33"/>
+      <c r="AF20" s="33"/>
+      <c r="AG20" s="33"/>
+      <c r="AH20" s="33"/>
+      <c r="AI20" s="33"/>
+      <c r="AJ20" s="33"/>
+      <c r="AK20" s="33"/>
+      <c r="AL20" s="34"/>
+      <c r="AM20" s="33"/>
+      <c r="AN20" s="33"/>
+      <c r="AO20" s="33"/>
+      <c r="AP20" s="33"/>
+      <c r="AQ20" s="33"/>
+      <c r="AR20" s="35"/>
       <c r="AS20" s="5"/>
     </row>
     <row r="21" spans="1:45" ht="15.75">
-      <c r="B21" s="73"/>
+      <c r="B21" s="25"/>
       <c r="C21" s="8"/>
       <c r="D21" s="8"/>
       <c r="E21" s="8"/>
@@ -2599,16 +2878,16 @@
       <c r="AI21" s="8"/>
       <c r="AJ21" s="8"/>
       <c r="AK21" s="8"/>
-      <c r="AL21" s="71"/>
+      <c r="AL21" s="23"/>
       <c r="AM21" s="8"/>
       <c r="AN21" s="8"/>
       <c r="AO21" s="8"/>
       <c r="AP21" s="8"/>
       <c r="AQ21" s="8"/>
-      <c r="AR21" s="71"/>
+      <c r="AR21" s="23"/>
     </row>
     <row r="22" spans="1:45" ht="15.75">
-      <c r="A22" s="71"/>
+      <c r="A22" s="23"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
@@ -5928,21 +6207,14 @@
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="U6:Y6"/>
-    <mergeCell ref="U7:Y7"/>
-    <mergeCell ref="U8:Y8"/>
-    <mergeCell ref="U9:Y9"/>
-    <mergeCell ref="AA6:AE6"/>
-    <mergeCell ref="AM8:AQ8"/>
-    <mergeCell ref="AM9:AQ9"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="O9:S9"/>
-    <mergeCell ref="B1:AR2"/>
-    <mergeCell ref="I4:M4"/>
-    <mergeCell ref="O4:S4"/>
-    <mergeCell ref="U4:Y4"/>
-    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="AG6:AK6"/>
+    <mergeCell ref="AG7:AK7"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="O6:S6"/>
+    <mergeCell ref="O7:S8"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="C13:G13"/>
     <mergeCell ref="C6:G6"/>
     <mergeCell ref="AM4:AQ4"/>
     <mergeCell ref="AM6:AQ6"/>
@@ -5951,15 +6223,592 @@
     <mergeCell ref="AA4:AE4"/>
     <mergeCell ref="AG4:AK4"/>
     <mergeCell ref="C10:G10"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="AG6:AK6"/>
-    <mergeCell ref="AG7:AK7"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="O6:S6"/>
-    <mergeCell ref="O7:S8"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="B1:AR2"/>
+    <mergeCell ref="I4:M4"/>
+    <mergeCell ref="O4:S4"/>
+    <mergeCell ref="U4:Y4"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="AM8:AQ8"/>
+    <mergeCell ref="AM9:AQ9"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="O9:S9"/>
+    <mergeCell ref="U6:Y6"/>
+    <mergeCell ref="U7:Y7"/>
+    <mergeCell ref="U8:Y8"/>
+    <mergeCell ref="U9:Y9"/>
+    <mergeCell ref="AA6:AE6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C30B422E-B08A-4402-AE47-DECD6D2FC0DE}">
+  <dimension ref="A1:H48"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="2.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="19.5">
+      <c r="A1" s="89" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="106" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="106"/>
+      <c r="G1" s="106"/>
+      <c r="H1" s="106"/>
+    </row>
+    <row r="2" spans="1:8" ht="19.5">
+      <c r="A2" s="107">
+        <v>1</v>
+      </c>
+      <c r="B2" s="108" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="108"/>
+      <c r="D2" s="108"/>
+    </row>
+    <row r="3" spans="1:8" ht="19.5">
+      <c r="A3" s="92"/>
+      <c r="B3" s="90" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="91" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="91"/>
+    </row>
+    <row r="4" spans="1:8" ht="19.5">
+      <c r="A4" s="92"/>
+      <c r="B4" s="92"/>
+      <c r="C4" s="90" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="90" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="19.5">
+      <c r="A5" s="92"/>
+      <c r="B5" s="92"/>
+      <c r="C5" s="90" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="90" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="19.5">
+      <c r="A6" s="92"/>
+      <c r="B6" s="92"/>
+      <c r="C6" s="90" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="90" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="19.5">
+      <c r="A7" s="92"/>
+      <c r="B7" s="92"/>
+      <c r="C7" s="90" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="90" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="19.5">
+      <c r="A8" s="92"/>
+      <c r="B8" s="92"/>
+      <c r="C8" s="90" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="90" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="19.5">
+      <c r="A9" s="92"/>
+      <c r="B9" s="90" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="91" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="91"/>
+    </row>
+    <row r="10" spans="1:8" ht="19.5">
+      <c r="A10" s="92"/>
+      <c r="B10" s="92"/>
+      <c r="C10" s="90" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="90" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="19.5">
+      <c r="A11" s="92"/>
+      <c r="B11" s="92"/>
+      <c r="C11" s="90" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="90" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="19.5">
+      <c r="A12" s="92"/>
+      <c r="B12" s="92"/>
+      <c r="C12" s="90" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="90" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="19.5">
+      <c r="A13" s="92"/>
+      <c r="B13" s="90" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="91" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="91"/>
+    </row>
+    <row r="14" spans="1:8" ht="19.5">
+      <c r="A14" s="92"/>
+      <c r="B14" s="92"/>
+      <c r="C14" s="90" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="90" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="19.5">
+      <c r="A15" s="92"/>
+      <c r="B15" s="92"/>
+      <c r="C15" s="90" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="90" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="19.5">
+      <c r="A16" s="92"/>
+      <c r="B16" s="92"/>
+      <c r="C16" s="90" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="90" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="19.5">
+      <c r="A17" s="92"/>
+      <c r="B17" s="92"/>
+      <c r="C17" s="90" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" s="90" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="19.5">
+      <c r="A18" s="92"/>
+      <c r="B18" s="92"/>
+      <c r="C18" s="90" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="90" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="19.5">
+      <c r="A19" s="92"/>
+      <c r="B19" s="92"/>
+      <c r="C19" s="90" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="90" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="19.5">
+      <c r="A20" s="109">
+        <v>2</v>
+      </c>
+      <c r="B20" s="110" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" s="110"/>
+      <c r="D20" s="110"/>
+    </row>
+    <row r="21" spans="1:4" ht="19.5">
+      <c r="A21" s="94"/>
+      <c r="B21" s="93" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21" s="121" t="s">
+        <v>61</v>
+      </c>
+      <c r="D21" s="121"/>
+    </row>
+    <row r="22" spans="1:4" ht="19.5">
+      <c r="A22" s="94"/>
+      <c r="B22" s="93" t="s">
+        <v>46</v>
+      </c>
+      <c r="C22" s="121" t="s">
+        <v>62</v>
+      </c>
+      <c r="D22" s="121"/>
+    </row>
+    <row r="23" spans="1:4" ht="19.5">
+      <c r="A23" s="94"/>
+      <c r="B23" s="93" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" s="121" t="s">
+        <v>63</v>
+      </c>
+      <c r="D23" s="121"/>
+    </row>
+    <row r="24" spans="1:4" ht="19.5">
+      <c r="A24" s="94"/>
+      <c r="B24" s="93" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="121" t="s">
+        <v>65</v>
+      </c>
+      <c r="D24" s="121"/>
+    </row>
+    <row r="25" spans="1:4" ht="19.5">
+      <c r="A25" s="94"/>
+      <c r="B25" s="93" t="s">
+        <v>66</v>
+      </c>
+      <c r="C25" s="121" t="s">
+        <v>67</v>
+      </c>
+      <c r="D25" s="121"/>
+    </row>
+    <row r="26" spans="1:4" ht="19.5">
+      <c r="A26" s="94"/>
+      <c r="B26" s="93" t="s">
+        <v>68</v>
+      </c>
+      <c r="C26" s="121" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" s="121"/>
+    </row>
+    <row r="27" spans="1:4" ht="19.5">
+      <c r="A27" s="94"/>
+      <c r="B27" s="93" t="s">
+        <v>70</v>
+      </c>
+      <c r="C27" s="121" t="s">
+        <v>71</v>
+      </c>
+      <c r="D27" s="121"/>
+    </row>
+    <row r="28" spans="1:4" ht="19.5">
+      <c r="A28" s="94"/>
+      <c r="B28" s="93" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" s="121" t="s">
+        <v>73</v>
+      </c>
+      <c r="D28" s="121"/>
+    </row>
+    <row r="29" spans="1:4" ht="19.5">
+      <c r="A29" s="111">
+        <v>3</v>
+      </c>
+      <c r="B29" s="112" t="s">
+        <v>74</v>
+      </c>
+      <c r="C29" s="112"/>
+      <c r="D29" s="112"/>
+    </row>
+    <row r="30" spans="1:4" ht="19.5">
+      <c r="A30" s="96"/>
+      <c r="B30" s="95" t="s">
+        <v>34</v>
+      </c>
+      <c r="C30" s="122" t="s">
+        <v>75</v>
+      </c>
+      <c r="D30" s="122"/>
+    </row>
+    <row r="31" spans="1:4" ht="19.5">
+      <c r="A31" s="96"/>
+      <c r="B31" s="95" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" s="122" t="s">
+        <v>76</v>
+      </c>
+      <c r="D31" s="122"/>
+    </row>
+    <row r="32" spans="1:4" ht="19.5">
+      <c r="A32" s="96"/>
+      <c r="B32" s="95" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="122" t="s">
+        <v>77</v>
+      </c>
+      <c r="D32" s="122"/>
+    </row>
+    <row r="33" spans="1:4" ht="19.5">
+      <c r="A33" s="113">
+        <v>4</v>
+      </c>
+      <c r="B33" s="114" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" s="114"/>
+      <c r="D33" s="114"/>
+    </row>
+    <row r="34" spans="1:4" ht="19.5">
+      <c r="A34" s="98"/>
+      <c r="B34" s="97" t="s">
+        <v>34</v>
+      </c>
+      <c r="C34" s="123" t="s">
+        <v>79</v>
+      </c>
+      <c r="D34" s="123"/>
+    </row>
+    <row r="35" spans="1:4" ht="19.5">
+      <c r="A35" s="98"/>
+      <c r="B35" s="97" t="s">
+        <v>46</v>
+      </c>
+      <c r="C35" s="123" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35" s="123"/>
+    </row>
+    <row r="36" spans="1:4" ht="19.5">
+      <c r="A36" s="98"/>
+      <c r="B36" s="97" t="s">
+        <v>51</v>
+      </c>
+      <c r="C36" s="123" t="s">
+        <v>81</v>
+      </c>
+      <c r="D36" s="123"/>
+    </row>
+    <row r="37" spans="1:4" ht="19.5">
+      <c r="A37" s="98"/>
+      <c r="B37" s="97" t="s">
+        <v>64</v>
+      </c>
+      <c r="C37" s="123" t="s">
+        <v>82</v>
+      </c>
+      <c r="D37" s="123"/>
+    </row>
+    <row r="38" spans="1:4" ht="19.5">
+      <c r="A38" s="98"/>
+      <c r="B38" s="97" t="s">
+        <v>66</v>
+      </c>
+      <c r="C38" s="123" t="s">
+        <v>83</v>
+      </c>
+      <c r="D38" s="123"/>
+    </row>
+    <row r="39" spans="1:4" ht="19.5">
+      <c r="A39" s="98"/>
+      <c r="B39" s="97" t="s">
+        <v>68</v>
+      </c>
+      <c r="C39" s="123" t="s">
+        <v>84</v>
+      </c>
+      <c r="D39" s="123"/>
+    </row>
+    <row r="40" spans="1:4" ht="19.5">
+      <c r="A40" s="98"/>
+      <c r="B40" s="97" t="s">
+        <v>70</v>
+      </c>
+      <c r="C40" s="123" t="s">
+        <v>85</v>
+      </c>
+      <c r="D40" s="123"/>
+    </row>
+    <row r="41" spans="1:4" ht="19.5">
+      <c r="A41" s="115">
+        <v>5</v>
+      </c>
+      <c r="B41" s="116" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41" s="116"/>
+      <c r="D41" s="116"/>
+    </row>
+    <row r="42" spans="1:4" ht="19.5">
+      <c r="A42" s="100"/>
+      <c r="B42" s="99" t="s">
+        <v>34</v>
+      </c>
+      <c r="C42" s="124" t="s">
+        <v>87</v>
+      </c>
+      <c r="D42" s="124"/>
+    </row>
+    <row r="43" spans="1:4" ht="19.5">
+      <c r="A43" s="100"/>
+      <c r="B43" s="99" t="s">
+        <v>46</v>
+      </c>
+      <c r="C43" s="124" t="s">
+        <v>88</v>
+      </c>
+      <c r="D43" s="124"/>
+    </row>
+    <row r="44" spans="1:4" ht="19.5">
+      <c r="A44" s="117">
+        <v>6</v>
+      </c>
+      <c r="B44" s="118" t="s">
+        <v>89</v>
+      </c>
+      <c r="C44" s="118"/>
+      <c r="D44" s="118"/>
+    </row>
+    <row r="45" spans="1:4" ht="19.5">
+      <c r="A45" s="103"/>
+      <c r="B45" s="101" t="s">
+        <v>34</v>
+      </c>
+      <c r="C45" s="102" t="s">
+        <v>90</v>
+      </c>
+      <c r="D45" s="102"/>
+    </row>
+    <row r="46" spans="1:4" ht="19.5">
+      <c r="A46" s="119">
+        <v>7</v>
+      </c>
+      <c r="B46" s="120" t="s">
+        <v>91</v>
+      </c>
+      <c r="C46" s="120"/>
+      <c r="D46" s="120"/>
+    </row>
+    <row r="47" spans="1:4" ht="19.5">
+      <c r="A47" s="105"/>
+      <c r="B47" s="104" t="s">
+        <v>34</v>
+      </c>
+      <c r="C47" s="125" t="s">
+        <v>92</v>
+      </c>
+      <c r="D47" s="125"/>
+    </row>
+    <row r="48" spans="1:4" ht="19.5">
+      <c r="A48" s="105"/>
+      <c r="B48" s="104" t="s">
+        <v>46</v>
+      </c>
+      <c r="C48" s="125" t="s">
+        <v>93</v>
+      </c>
+      <c r="D48" s="125"/>
+    </row>
+  </sheetData>
+  <mergeCells count="34">
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C30:D30"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4530DDDC-9A48-4BD8-8919-C60744941AAD}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>